<commit_message>
Adding files from Mac for GEMINI Archive
</commit_message>
<xml_diff>
--- a/GEMINI-Data/GEMINI_FirstLightTestPlan.xlsx
+++ b/GEMINI-Data/GEMINI_FirstLightTestPlan.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{8701781B-65B4-4540-B020-9EF91FB75FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="2" xr2:uid="{238EBA84-722F-2142-A8CD-6FA9A1539EDF}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="1" xr2:uid="{238EBA84-722F-2142-A8CD-6FA9A1539EDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Day 1 Test Plan" sheetId="10" r:id="rId1"/>
@@ -2244,10 +2244,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -16064,21 +16060,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010001B84A3B81A43243B60565715F143EA4" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dcab34dfa5210f6f5692f5b7ea2c33f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="a48f74a4-b394-405e-8217-14c7a0c9c8dd" xmlns:ns4="ad2059a1-cba4-4d67-9ee9-c16ee1049fd9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="039b9c5d034462043671331dd9f3c14d" ns3:_="" ns4:_="">
     <xsd:import namespace="a48f74a4-b394-405e-8217-14c7a0c9c8dd"/>
@@ -16301,10 +16282,36 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A662B9C4-A5A2-4999-B3B5-B87F26ABA290}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5C2C3F8-F2EC-45A3-966B-4E284025B674}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a48f74a4-b394-405e-8217-14c7a0c9c8dd"/>
+    <ds:schemaRef ds:uri="ad2059a1-cba4-4d67-9ee9-c16ee1049fd9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -16327,20 +16334,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5C2C3F8-F2EC-45A3-966B-4E284025B674}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A662B9C4-A5A2-4999-B3B5-B87F26ABA290}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="a48f74a4-b394-405e-8217-14c7a0c9c8dd"/>
-    <ds:schemaRef ds:uri="ad2059a1-cba4-4d67-9ee9-c16ee1049fd9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>